<commit_message>
Display physician counts as integers
</commit_message>
<xml_diff>
--- a/OPD_test_instances.xlsx
+++ b/OPD_test_instances.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" r:id="R5e2ebf8230e24b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" r:id="Ra011a797a9e64af0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,8 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -46,13 +47,14 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -371,7 +373,7 @@
       <x:c r="A2" s="1" t="str">
         <x:v>s-1</x:v>
       </x:c>
-      <x:c r="B2" s="3" t="n">
+      <x:c r="B2" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C2" s="3" t="n">
@@ -446,7 +448,7 @@
       <x:c r="A3" s="1" t="str">
         <x:v>s-2</x:v>
       </x:c>
-      <x:c r="B3" s="3" t="n">
+      <x:c r="B3" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C3" s="3" t="n">
@@ -521,7 +523,7 @@
       <x:c r="A4" s="1" t="str">
         <x:v>s-3</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="n">
+      <x:c r="B4" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="3" t="n">
@@ -596,7 +598,7 @@
       <x:c r="A5" s="1" t="str">
         <x:v>s-4</x:v>
       </x:c>
-      <x:c r="B5" s="3" t="n">
+      <x:c r="B5" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C5" s="3" t="n">
@@ -671,7 +673,7 @@
       <x:c r="A6" s="1" t="str">
         <x:v>s-5</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="n">
+      <x:c r="B6" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="3" t="n">
@@ -746,7 +748,7 @@
       <x:c r="A7" s="1" t="str">
         <x:v>s-6</x:v>
       </x:c>
-      <x:c r="B7" s="3" t="n">
+      <x:c r="B7" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="3" t="n">
@@ -821,7 +823,7 @@
       <x:c r="A8" s="1" t="str">
         <x:v>o-1</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="n">
+      <x:c r="B8" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C8" s="3" t="n">
@@ -904,7 +906,7 @@
       <x:c r="A9" s="1" t="str">
         <x:v>o-2</x:v>
       </x:c>
-      <x:c r="B9" s="3" t="n">
+      <x:c r="B9" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C9" s="3" t="n">
@@ -987,7 +989,7 @@
       <x:c r="A10" s="1" t="str">
         <x:v>o-3</x:v>
       </x:c>
-      <x:c r="B10" s="3" t="n">
+      <x:c r="B10" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C10" s="3" t="n">
@@ -1070,7 +1072,7 @@
       <x:c r="A11" s="1" t="str">
         <x:v>o-4</x:v>
       </x:c>
-      <x:c r="B11" s="3" t="n">
+      <x:c r="B11" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C11" s="3" t="n">
@@ -1153,7 +1155,7 @@
       <x:c r="A12" s="1" t="str">
         <x:v>o-5</x:v>
       </x:c>
-      <x:c r="B12" s="3" t="n">
+      <x:c r="B12" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C12" s="3" t="n">
@@ -1236,7 +1238,7 @@
       <x:c r="A13" s="1" t="str">
         <x:v>o-6</x:v>
       </x:c>
-      <x:c r="B13" s="3" t="n">
+      <x:c r="B13" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C13" s="3" t="n">

</xml_diff>